<commit_message>
feat: put building_construction_end_date as recommended
</commit_message>
<xml_diff>
--- a/translators/translator_template.xlsx
+++ b/translators/translator_template.xlsx
@@ -4020,9 +4020,9 @@
           <t>date</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>Required</t>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr"/>

</xml_diff>